<commit_message>
fix: grammar audit pass 1 — 62 corrections across L1–L5
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/grammar.xlsx
+++ b/grammar.xlsx
@@ -1370,12 +1370,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>这个电影很好，也非常好看，你看看吧。</t>
+          <t>这个苹果很好，也非常好吃，你吃吃吧。</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>This movie is very good and also really great to watch — watch it.</t>
+          <t>This apple is very good and also really delicious — have a taste.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>你会说中文，他也会，还会说英语。</t>
+          <t>你会说中文，他也会，还会写汉字。</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>You can speak Chinese; he can too, and he can also speak English.</t>
+          <t>You can speak Chinese; he can too, and he can also write Chinese characters.</t>
         </is>
       </c>
     </row>
@@ -2491,12 +2491,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>他在家学习汉语。</t>
+          <t>他给妈妈打电话了。</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>He studies Chinese at home.</t>
+          <t>He called his mom.</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>电影很好看。</t>
+          <t>电视很好看。</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3883,12 +3883,12 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>他去商店买东西。</t>
+          <t>她去医院看病。</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>He went to the shop to buy things.</t>
+          <t>She went to the hospital to see the doctor.</t>
         </is>
       </c>
     </row>
@@ -4235,12 +4235,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>我吃了早饭，去学校了。</t>
+          <t>我吃了一个苹果。</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>I ate breakfast and went to school.</t>
+          <t>I ate an apple.</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4872,12 +4872,12 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>你看一看这件衣服，喜欢吗？</t>
+          <t>你们休息休息吧，走了这么长时间了。</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Have a look at this piece of clothing — do you like it?</t>
+          <t>Rest for a bit — you've been walking for so long.</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5006,12 +5006,12 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>他喜欢跑步，每天早上跑半个小时步。</t>
+          <t>她昨天跳了一个晚上舞，很累。</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>He likes running and runs for half an hour every morning.</t>
+          <t>She danced the whole evening yesterday and is very tired.</t>
         </is>
       </c>
     </row>
@@ -5172,12 +5172,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>你这样做是对的。</t>
+          <t>今天这么热，我不想出去。</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Doing it this way is correct.</t>
+          <t>It's so hot today — I don't want to go out.</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5673,12 +5673,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>我正在吃饭，饭已经好了，你来吧。</t>
+          <t>饭已经好了，你快来吧。</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>I'm eating; the food is already ready — come on over.</t>
+          <t>The food is already ready — hurry and come over.</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6551,12 +6551,12 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>她高兴地唱歌。</t>
+          <t>她慢慢地走进教室。</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>She sings happily.</t>
+          <t>She walked slowly into the classroom.</t>
         </is>
       </c>
     </row>
@@ -7597,12 +7597,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>学了一年，我学会唱这首歌了。</t>
+          <t>老师说的话，我听懂了。</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>After studying for a year, I learned to sing this song.</t>
+          <t>I understood what the teacher said.</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -7711,12 +7711,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>他跑出了房间，去找妈妈。</t>
+          <t>他跑上楼去找妈妈。</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>He ran out of the room to find his mom.</t>
+          <t>He ran upstairs to find his mom.</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7731,12 +7731,12 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>他跑出了教室，没有回来。</t>
+          <t>她走过去，把书给了他。</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>He ran out of the classroom and didn't come back.</t>
+          <t>She walked over and gave him the book.</t>
         </is>
       </c>
     </row>
@@ -9194,12 +9194,12 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>我从来没坐过地铁。</t>
+          <t>我没有坐过飞机。</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>I have never taken the subway.</t>
+          <t>I have never been on a plane.</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9670,12 +9670,12 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>你需要多休息，明天还得上班呢。</t>
+          <t>他愿意帮忙，你不必担心。</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>You need to rest more — you still have to go to work tomorrow.</t>
+          <t>He is willing to help — you don't need to worry.</t>
         </is>
       </c>
     </row>
@@ -9712,12 +9712,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>他们打算明年结婚，已经开始准备了。</t>
+          <t>他们上个月见了一次面，觉得很开心。</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>They plan to get married next year and have already started preparing.</t>
+          <t>They met up once last month and had a great time.</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9794,12 +9794,12 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>他们完成了作业，高兴地分开了。</t>
+          <t>作业太多了，我今天完不成。</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>They finished the homework and happily went their separate ways.</t>
+          <t>There's too much homework — I can't finish it today.</t>
         </is>
       </c>
     </row>
@@ -11282,12 +11282,12 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>如果你有时间，我们吃完饭然后一起去公园吧。</t>
+          <t>你只有多练习，才能说好汉语。</t>
         </is>
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>If you have time, let's go to the park together after dinner.</t>
+          <t>Only by practicing more can you speak Chinese well.</t>
         </is>
       </c>
     </row>
@@ -11468,12 +11468,12 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>他跑得太快了，我跟不上。</t>
+          <t>这道菜好吃极了，我又吃了一碗。</t>
         </is>
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>He runs too fast — I can't keep up.</t>
+          <t>This dish is extremely delicious — I had another bowl.</t>
         </is>
       </c>
     </row>
@@ -12722,12 +12722,12 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>他工作很努力，这让大家都很高兴。</t>
+          <t>他每天努力工作让大家很高兴。</t>
         </is>
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>He works very hard — this makes everyone very happy.</t>
+          <t>His working hard every day makes everyone very happy.</t>
         </is>
       </c>
     </row>
@@ -12841,12 +12841,12 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>他把书放上了桌子。</t>
+          <t>他的钱包被人拿走了。</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>He put the book on the table.</t>
+          <t>His wallet was taken away by someone.</t>
         </is>
       </c>
     </row>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>When they heard he was back, everyone started to cheer up.</t>
+          <t>When they heard he was back, everyone started to get happy.</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -14681,12 +14681,12 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>不但我学中文，我弟弟也学中文。</t>
+          <t>不但我学中文，而且我弟弟也学中文。</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>Not only do I study Chinese, my younger brother does too.</t>
+          <t>Not only do I study Chinese, but my younger brother does too.</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15492,12 +15492,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>他跑步回来，脸上一脸汗，手上也是一手水。</t>
+          <t>他跑步回来，一脸汗，手上也是一手汗。</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>When he came back, his face was dripping with sweat and his hands were covered in water.</t>
+          <t>When he came back, his face was dripping with sweat and his hands were covered in sweat too.</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -17228,12 +17228,12 @@
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>他总找借口，这就是说他不想负责任。</t>
+          <t>他总是说没时间，这就是说他不想参加。</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>He always makes excuses — in other words, he doesn't want to take responsibility.</t>
+          <t>He always says he has no time — in other words, he doesn't want to participate.</t>
         </is>
       </c>
     </row>
@@ -19498,12 +19498,12 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>我经常去健身房，甚至还请了健身教练。</t>
+          <t>我经常去健身房，甚至还请了教练。</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>I go to the gym regularly — I even hired a personal trainer.</t>
+          <t>I go to the gym regularly — I even hired a trainer.</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -19580,12 +19580,12 @@
       </c>
       <c r="K318" t="inlineStr">
         <is>
-          <t>她不仅会说汉语，还会说法语和西班牙语。</t>
+          <t>她不仅会说汉语，还会说别的外语。</t>
         </is>
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>She can not only speak Chinese but also French and Spanish.</t>
+          <t>She can not only speak Chinese but also other foreign languages.</t>
         </is>
       </c>
     </row>
@@ -19684,12 +19684,12 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>她连简单的问候都说不好，更难说整段对话了。</t>
+          <t>她连简单的打招呼都说不好，更难说整个对话了。</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>She can't even manage a simple greeting well, let alone a whole conversation.</t>
+          <t>She can't even manage a simple greeting well, let alone an entire conversation.</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -19756,12 +19756,12 @@
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>周末他不是在游泳馆游泳，就是在篮球场打篮球。</t>
+          <t>周末他不是去游泳，就是在球场打篮球。</t>
         </is>
       </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>On weekends he is either swimming at the pool or playing basketball on the court.</t>
+          <t>On weekends he is either swimming or playing basketball on the court.</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
@@ -22040,12 +22040,12 @@
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t>你同他一起去吧，路上有个伴。</t>
+          <t>老师同家长都参加了这次家长会。</t>
         </is>
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>Go together with him — you'll have company on the way.</t>
+          <t>Both the teachers and the parents attended the parent-teacher meeting.</t>
         </is>
       </c>
     </row>
@@ -22092,12 +22092,12 @@
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>假如你有时间，可以来参加我们的活动。</t>
+          <t>他每天坚持练习，可见他非常热爱这项运动。</t>
         </is>
       </c>
       <c r="J359" t="inlineStr">
         <is>
-          <t>If you have time, you are welcome to join our event.</t>
+          <t>He practises every day — it is clear he is very passionate about this activity.</t>
         </is>
       </c>
       <c r="K359" t="inlineStr">

</xml_diff>